<commit_message>
update hyperparameters for better val loss
</commit_message>
<xml_diff>
--- a/Plots/average_results.xlsx
+++ b/Plots/average_results.xlsx
@@ -482,22 +482,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.8758064516129032</v>
+        <v>0.8463058183553649</v>
       </c>
       <c r="D2" t="n">
-        <v>0.004017040197077555</v>
+        <v>0.008931327843261399</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8756360843189285</v>
+        <v>0.8720839328663378</v>
       </c>
       <c r="F2" t="n">
-        <v>0.003996550101957328</v>
+        <v>0.02318794761986417</v>
       </c>
       <c r="G2" t="n">
-        <v>22.18402705515089</v>
+        <v>21.42220618575556</v>
       </c>
       <c r="H2" t="n">
-        <v>0.108347112980168</v>
+        <v>2.201746111821201</v>
       </c>
     </row>
     <row r="3">
@@ -512,22 +512,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.8741098677517802</v>
+        <v>0.8458853863632081</v>
       </c>
       <c r="D3" t="n">
-        <v>0.00389538596104697</v>
+        <v>0.003201486021015792</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8739844062024383</v>
+        <v>0.8695998255514302</v>
       </c>
       <c r="F3" t="n">
-        <v>0.003776075454863565</v>
+        <v>0.0218453198916433</v>
       </c>
       <c r="G3" t="n">
-        <v>22.28021363173957</v>
+        <v>21.32778107182569</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1013141193074419</v>
+        <v>2.424561132462312</v>
       </c>
     </row>
     <row r="4">
@@ -542,22 +542,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.8806338028169014</v>
+        <v>0.7477963697499246</v>
       </c>
       <c r="D4" t="n">
-        <v>0.004632411718246577</v>
+        <v>0.04010031161698811</v>
       </c>
       <c r="E4" t="n">
-        <v>0.8807231679213006</v>
+        <v>0.7871335118966196</v>
       </c>
       <c r="F4" t="n">
-        <v>0.004665816329712545</v>
+        <v>0.02874702591219274</v>
       </c>
       <c r="G4" t="n">
-        <v>23.837144339651</v>
+        <v>28.16084181865457</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1840530226859428</v>
+        <v>1.530532679221874</v>
       </c>
     </row>
     <row r="5">
@@ -572,22 +572,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.8772</v>
+        <v>0.752781746031746</v>
       </c>
       <c r="D5" t="n">
-        <v>0.005254521862167833</v>
+        <v>0.01589977357774736</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8775443969011849</v>
+        <v>0.7872744341695569</v>
       </c>
       <c r="F5" t="n">
-        <v>0.00518060220485561</v>
+        <v>0.03103278447963139</v>
       </c>
       <c r="G5" t="n">
-        <v>23.44439355165616</v>
+        <v>28.92131158172477</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2083238937955884</v>
+        <v>1.209140664408459</v>
       </c>
     </row>
   </sheetData>

</xml_diff>